<commit_message>
Pizza Sales Data Analysis (Python) Group commit
</commit_message>
<xml_diff>
--- a/Python_Projects/Pizza_Sales_Data_Analysis/2_Descriptive_Sales_Analysis/Assets/Descriptive_Sales_Analysis_Excel.xlsx
+++ b/Python_Projects/Pizza_Sales_Data_Analysis/2_Descriptive_Sales_Analysis/Assets/Descriptive_Sales_Analysis_Excel.xlsx
@@ -1371,6 +1371,2989 @@
 </styleSheet>
 </file>
 
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>133355</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>30488</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1" descr="Top 10 Pizza IDs (T S)_hbar_count.png"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="514350" y="3048000"/>
+          <a:ext cx="2743205" cy="3840488"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>314330</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>30488</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2" descr="Top 10 Pizza IDs (T S)_hbar_pct_count.png"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3124200" y="3048000"/>
+          <a:ext cx="2743205" cy="3840488"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>314330</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>30488</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 3" descr="Top 10 Pizza IDs (T S)_hbar_total_sales.png"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="7067550" y="3048000"/>
+          <a:ext cx="2743205" cy="3840488"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>1228730</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>30488</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Picture 4" descr="Top 10 Pizza IDs (T S)_hbar_pct_total_sales.png"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="10410825" y="3048000"/>
+          <a:ext cx="2743205" cy="3840488"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing10.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>47630</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>30488</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1" descr="Top 10 Names (C)_hbar_count.png"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="514350" y="3048000"/>
+          <a:ext cx="2743205" cy="3840488"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>314330</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>30488</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2" descr="Top 10 Names (C)_hbar_pct_count.png"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4124325" y="3048000"/>
+          <a:ext cx="2743205" cy="3840488"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>314330</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>30488</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 3" descr="Top 10 Names (C)_hbar_total_sales.png"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="8201025" y="3048000"/>
+          <a:ext cx="2743205" cy="3840488"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>1228730</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>30488</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Picture 4" descr="Top 10 Names (C)_hbar_pct_total_sales.png"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="11544300" y="3048000"/>
+          <a:ext cx="2743205" cy="3840488"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing11.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>47630</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>30488</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1" descr="Bottom 10 Names (T S)_hbar_count.png"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="514350" y="3048000"/>
+          <a:ext cx="2743205" cy="3840488"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>314330</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>30488</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2" descr="Bottom 10 Names (T S)_hbar_pct_count.png"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4124325" y="3048000"/>
+          <a:ext cx="2743205" cy="3840488"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>314330</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>30488</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 3" descr="Bottom 10 Names (T S)_hbar_total_sales.png"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="8134350" y="3048000"/>
+          <a:ext cx="2743205" cy="3840488"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>1228730</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>30488</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Picture 4" descr="Bottom 10 Names (T S)_hbar_pct_total_sales.png"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="11477625" y="3048000"/>
+          <a:ext cx="2743205" cy="3840488"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing12.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>47630</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>30488</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1" descr="Bottom 10 Names (C)_hbar_count.png"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="514350" y="3048000"/>
+          <a:ext cx="2743205" cy="3840488"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>314330</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>30488</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2" descr="Bottom 10 Names (C)_hbar_pct_count.png"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4124325" y="3048000"/>
+          <a:ext cx="2743205" cy="3840488"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>314330</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>30488</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 3" descr="Bottom 10 Names (C)_hbar_total_sales.png"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="8134350" y="3048000"/>
+          <a:ext cx="2743205" cy="3840488"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>1228730</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>30488</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Picture 4" descr="Bottom 10 Names (C)_hbar_pct_total_sales.png"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="11477625" y="3048000"/>
+          <a:ext cx="2743205" cy="3840488"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing13.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>466730</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>30488</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1" descr="Top Categories (T S)_hbar_count.png"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="514350" y="1905000"/>
+          <a:ext cx="2743205" cy="3840488"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>314330</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>30488</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2" descr="Top Categories (T S)_hbar_pct_count.png"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2790825" y="1905000"/>
+          <a:ext cx="2743205" cy="3840488"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>314330</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>30488</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 3" descr="Top Categories (T S)_hbar_total_sales.png"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6734175" y="1905000"/>
+          <a:ext cx="2743205" cy="3840488"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>1228730</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>30488</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Picture 4" descr="Top Categories (T S)_hbar_pct_total_sales.png"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="10077450" y="1905000"/>
+          <a:ext cx="2743205" cy="3840488"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing14.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>733430</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>30488</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1" descr="Top Sizes (T S)_hbar_count.png"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="514350" y="2095500"/>
+          <a:ext cx="2743205" cy="3840488"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>180980</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>30488</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2" descr="Top Sizes (T S)_hbar_pct_count.png"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2524125" y="2095500"/>
+          <a:ext cx="2743205" cy="3840488"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>1295405</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>30488</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 3" descr="Top Sizes (T S)_hbar_total_sales.png"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6600825" y="2095500"/>
+          <a:ext cx="2743205" cy="3840488"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>1095380</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>30488</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Picture 4" descr="Top Sizes (T S)_hbar_pct_total_sales.png"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="10410825" y="2095500"/>
+          <a:ext cx="2743205" cy="3840488"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing15.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>400055</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>30488</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1" descr="Top Days_hbar_count.png"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="514350" y="2476500"/>
+          <a:ext cx="2743205" cy="3840488"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>314330</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>30488</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2" descr="Top Days_hbar_pct_count.png"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2857500" y="2476500"/>
+          <a:ext cx="2743205" cy="3840488"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>314330</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>30488</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 3" descr="Top Days_hbar_total_sales.png"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6800850" y="2476500"/>
+          <a:ext cx="2743205" cy="3840488"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>1228730</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>30488</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Picture 4" descr="Top Days_hbar_pct_total_sales.png"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="10144125" y="2476500"/>
+          <a:ext cx="2743205" cy="3840488"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing16.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>400055</xdr:colOff>
+      <xdr:row>38</xdr:row>
+      <xdr:rowOff>30488</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1" descr="Top Months_hbar_count.png"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="514350" y="3429000"/>
+          <a:ext cx="2743205" cy="3840488"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>314330</xdr:colOff>
+      <xdr:row>38</xdr:row>
+      <xdr:rowOff>30488</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2" descr="Top Months_hbar_pct_count.png"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2857500" y="3429000"/>
+          <a:ext cx="2743205" cy="3840488"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>314330</xdr:colOff>
+      <xdr:row>38</xdr:row>
+      <xdr:rowOff>30488</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 3" descr="Top Months_hbar_total_sales.png"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6800850" y="3429000"/>
+          <a:ext cx="2743205" cy="3840488"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>1228730</xdr:colOff>
+      <xdr:row>38</xdr:row>
+      <xdr:rowOff>30488</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Picture 4" descr="Top Months_hbar_pct_total_sales.png"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="10144125" y="3429000"/>
+          <a:ext cx="2743205" cy="3840488"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing17.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>533405</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>30488</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1" descr="Top Quarters_hbar_count.png"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="514350" y="1905000"/>
+          <a:ext cx="2743205" cy="3840488"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>314330</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>30488</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2" descr="Top Quarters_hbar_pct_count.png"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2724150" y="1905000"/>
+          <a:ext cx="2743205" cy="3840488"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>1295405</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>30488</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 3" descr="Top Quarters_hbar_total_sales.png"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6667500" y="1905000"/>
+          <a:ext cx="2743205" cy="3840488"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>1228730</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>30488</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Picture 4" descr="Top Quarters_hbar_pct_total_sales.png"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="10410825" y="1905000"/>
+          <a:ext cx="2743205" cy="3840488"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing18.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>133355</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>30488</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1" descr="Top Quarter Labels_hbar_count.png"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="514350" y="1905000"/>
+          <a:ext cx="2743205" cy="3840488"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>314330</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>30488</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2" descr="Top Quarter Labels_hbar_pct_count.png"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3124200" y="1905000"/>
+          <a:ext cx="2743205" cy="3840488"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>1295405</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>30488</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 3" descr="Top Quarter Labels_hbar_total_sales.png"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="7067550" y="1905000"/>
+          <a:ext cx="2743205" cy="3840488"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>1228730</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>30488</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Picture 4" descr="Top Quarter Labels_hbar_pct_total_sales.png"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="10810875" y="1905000"/>
+          <a:ext cx="2743205" cy="3840488"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing19.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>733430</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>30488</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1" descr="Top Years_hbar_count.png"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="514350" y="1333500"/>
+          <a:ext cx="2743205" cy="3840488"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>981080</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>30488</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2" descr="Top Years_hbar_pct_count.png"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2524125" y="1333500"/>
+          <a:ext cx="2743205" cy="3840488"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>314330</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>30488</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 3" descr="Top Years_hbar_total_sales.png"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5467350" y="1333500"/>
+          <a:ext cx="2743205" cy="3840488"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>180980</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>30488</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Picture 4" descr="Top Years_hbar_pct_total_sales.png"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="8810625" y="1333500"/>
+          <a:ext cx="2743205" cy="3840488"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>133355</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>30488</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1" descr="Top 10 Pizza IDs (C)_hbar_count.png"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="514350" y="3048000"/>
+          <a:ext cx="2743205" cy="3840488"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>314330</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>30488</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2" descr="Top 10 Pizza IDs (C)_hbar_pct_count.png"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3124200" y="3048000"/>
+          <a:ext cx="2743205" cy="3840488"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>314330</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>30488</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 3" descr="Top 10 Pizza IDs (C)_hbar_total_sales.png"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="7067550" y="3048000"/>
+          <a:ext cx="2743205" cy="3840488"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>1228730</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>30488</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Picture 4" descr="Top 10 Pizza IDs (C)_hbar_pct_total_sales.png"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="10410825" y="3048000"/>
+          <a:ext cx="2743205" cy="3840488"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>66680</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>30488</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1" descr="Bottom 10 Pizza IDs (T S)_hbar_count.png"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="514350" y="3048000"/>
+          <a:ext cx="2743205" cy="3840488"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>247655</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>30488</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2" descr="Bottom 10 Pizza IDs (T S)_hbar_pct_count.png"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3190875" y="3048000"/>
+          <a:ext cx="2743205" cy="3840488"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>1295405</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>30488</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 3" descr="Bottom 10 Pizza IDs (T S)_hbar_total_sales.png"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="7200900" y="3048000"/>
+          <a:ext cx="2743205" cy="3840488"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>1162055</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>30488</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Picture 4" descr="Bottom 10 Pizza IDs (T S)_hbar_pct_total_sales.png"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="11010900" y="3048000"/>
+          <a:ext cx="2743205" cy="3840488"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>66680</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>30488</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1" descr="Bottom 10 Pizza IDs (C)_hbar_count.png"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="514350" y="3048000"/>
+          <a:ext cx="2743205" cy="3840488"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>247655</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>30488</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2" descr="Bottom 10 Pizza IDs (C)_hbar_pct_count.png"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3190875" y="3048000"/>
+          <a:ext cx="2743205" cy="3840488"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>1295405</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>30488</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 3" descr="Bottom 10 Pizza IDs (C)_hbar_total_sales.png"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="7200900" y="3048000"/>
+          <a:ext cx="2743205" cy="3840488"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>1228730</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>30488</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Picture 4" descr="Bottom 10 Pizza IDs (C)_hbar_pct_total_sales.png"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="11010900" y="3048000"/>
+          <a:ext cx="2743205" cy="3840488"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>133355</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>30488</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1" descr="Top 10 Pizza Type IDs (T S)_hbar_count.png"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="514350" y="3048000"/>
+          <a:ext cx="2743205" cy="3840488"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>314330</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>30488</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2" descr="Top 10 Pizza Type IDs (T S)_hbar_pct_count.png"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3124200" y="3048000"/>
+          <a:ext cx="2743205" cy="3840488"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>314330</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>30488</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 3" descr="Top 10 Pizza Type IDs (T S)_hbar_total_sales.png"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="7134225" y="3048000"/>
+          <a:ext cx="2743205" cy="3840488"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>1228730</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>30488</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Picture 4" descr="Top 10 Pizza Type IDs (T S)_hbar_pct_total_sales.png"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="10477500" y="3048000"/>
+          <a:ext cx="2743205" cy="3840488"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>133355</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>30488</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1" descr="Top 10 Pizza Type IDs (C)_hbar_count.png"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="514350" y="3048000"/>
+          <a:ext cx="2743205" cy="3840488"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>314330</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>30488</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2" descr="Top 10 Pizza Type IDs (C)_hbar_pct_count.png"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3124200" y="3048000"/>
+          <a:ext cx="2743205" cy="3840488"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>314330</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>30488</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 3" descr="Top 10 Pizza Type IDs (C)_hbar_total_sales.png"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="7200900" y="3048000"/>
+          <a:ext cx="2743205" cy="3840488"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>1228730</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>30488</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Picture 4" descr="Top 10 Pizza Type IDs (C)_hbar_pct_total_sales.png"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="10544175" y="3048000"/>
+          <a:ext cx="2743205" cy="3840488"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing7.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>133355</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>30488</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1" descr="Bottom 10 Pizza Type IDs (T S)_hbar_count.png"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="514350" y="3048000"/>
+          <a:ext cx="2743205" cy="3840488"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>314330</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>30488</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2" descr="Bottom 10 Pizza Type IDs (T S)_hbar_pct_count.png"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3124200" y="3048000"/>
+          <a:ext cx="2743205" cy="3840488"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>314330</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>30488</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 3" descr="Bottom 10 Pizza Type IDs (T S)_hbar_total_sales.png"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="7134225" y="3048000"/>
+          <a:ext cx="2743205" cy="3840488"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>1228730</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>30488</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Picture 4" descr="Bottom 10 Pizza Type IDs (T S)_hbar_pct_total_sales.png"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="10477500" y="3048000"/>
+          <a:ext cx="2743205" cy="3840488"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing8.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>133355</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>30488</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1" descr="Bottom 10 Pizza Type IDs (C)_hbar_count.png"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="514350" y="3048000"/>
+          <a:ext cx="2743205" cy="3840488"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>314330</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>30488</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2" descr="Bottom 10 Pizza Type IDs (C)_hbar_pct_count.png"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3124200" y="3048000"/>
+          <a:ext cx="2743205" cy="3840488"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>314330</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>30488</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 3" descr="Bottom 10 Pizza Type IDs (C)_hbar_total_sales.png"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="7134225" y="3048000"/>
+          <a:ext cx="2743205" cy="3840488"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>1228730</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>30488</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Picture 4" descr="Bottom 10 Pizza Type IDs (C)_hbar_pct_total_sales.png"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="10477500" y="3048000"/>
+          <a:ext cx="2743205" cy="3840488"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing9.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>47630</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>30488</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1" descr="Top 10 Names (T S)_hbar_count.png"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="514350" y="3048000"/>
+          <a:ext cx="2743205" cy="3840488"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>314330</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>30488</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2" descr="Top 10 Names (T S)_hbar_pct_count.png"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4124325" y="3048000"/>
+          <a:ext cx="2743205" cy="3840488"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>314330</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>30488</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 3" descr="Top 10 Names (T S)_hbar_total_sales.png"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="8134350" y="3048000"/>
+          <a:ext cx="2743205" cy="3840488"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>1228730</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>30488</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Picture 4" descr="Top 10 Names (T S)_hbar_pct_total_sales.png"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="11477625" y="3048000"/>
+          <a:ext cx="2743205" cy="3840488"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -2249,6 +5232,7 @@
     <mergeCell ref="A1:N1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -2847,6 +5831,7 @@
     <mergeCell ref="A1:N1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -3446,6 +6431,7 @@
     <mergeCell ref="A1:N1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -4045,6 +7031,7 @@
     <mergeCell ref="A1:N1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -4361,6 +7348,7 @@
     <mergeCell ref="A1:N1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -4723,6 +7711,7 @@
     <mergeCell ref="A1:N1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -5180,6 +8169,7 @@
     <mergeCell ref="A1:N1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -5872,6 +8862,7 @@
     <mergeCell ref="A1:N1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -6188,6 +9179,7 @@
     <mergeCell ref="A1:N1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -6504,6 +9496,7 @@
     <mergeCell ref="A1:N1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -6679,6 +9672,7 @@
     <mergeCell ref="A1:N1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -7277,6 +10271,7 @@
     <mergeCell ref="A1:N1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -7875,6 +10870,7 @@
     <mergeCell ref="A1:N1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -8473,6 +11469,7 @@
     <mergeCell ref="A1:N1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -9071,6 +12068,7 @@
     <mergeCell ref="A1:N1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -9669,6 +12667,7 @@
     <mergeCell ref="A1:N1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -10268,6 +13267,7 @@
     <mergeCell ref="A1:N1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -10867,6 +13867,7 @@
     <mergeCell ref="A1:N1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -11465,5 +14466,6 @@
     <mergeCell ref="A1:N1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>